<commit_message>
[feat] - Completar escenarios de Venta cotidiana y su cobertura
Implementar XG-VEN-003 a XG-VEN-009 para editar cantidades, rechazar códigos inexistentes, cobrar con vuelto, cancelar y retomar cobros y continuar después de cobrar o abandonar. Exigir la extensión calibrada ventas-etapa1 antes de iniciar los nuevos recorridos.

Actualizar fichas, README, roadmap y Excel a 14 escenarios implementados, conservando la validación real sobre el JAR como pendiente. Registrar en el backlog CSV la mejora para abrir el editor por teclado y cubrir contratos, continuidad y diagnósticos con pruebas sintéticas.

Validación: 419 tests del framework aprobados y 34 omitidos; Ruff, Robocop, catálogo, mapa de cobertura y dry-run de los 14 casos correctos. Calibración y aceptación sobre el paquete privado pendientes.
</commit_message>
<xml_diff>
--- a/docs/coverage/xgestion-cobertura.xlsx
+++ b/docs/coverage/xgestion-cobertura.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R92a76bd6280b415f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="2" r:id="Rfcd166cfe98e4592"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenarios" sheetId="3" r:id="R7f13a62c8c464ea5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por detallar" sheetId="4" r:id="Rdb44edbfdb47449b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplos seed" sheetId="5" r:id="Re8eb3434e3004eaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R93a9a537d9eb4d92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="2" r:id="R6c55d5c238a74a25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenarios" sheetId="3" r:id="R963b9572bf9a4b8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por detallar" sheetId="4" r:id="Rfbea94cef47a4a5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplos seed" sheetId="5" r:id="R5153ee3f4c0342fc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -523,7 +523,7 @@
       </x:c>
       <x:c r="B8" s="21" t="n">
         <x:f>COUNTIF('Escenarios'!$C$7:$C$20,"Automatizado")</x:f>
-        <x:v>7</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C8" s="3" t="str">
         <x:v>Código de prueba disponible. Ejecución real pendiente.</x:v>
@@ -535,7 +535,7 @@
       </x:c>
       <x:c r="B9" s="22" t="n">
         <x:f>COUNTIF('Escenarios'!$C$7:$C$20,"Pendiente")</x:f>
-        <x:v>7</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
         <x:v>Criterios escritos; todavía sin prueba ejecutable.</x:v>
@@ -667,10 +667,10 @@
         <x:v>1. Venta cotidiana</x:v>
       </x:c>
       <x:c r="B23" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C23" s="3" t="str">
-        <x:v>7 pendientes · 0 manuales</x:v>
+        <x:v>0 pendientes · 0 manuales</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
@@ -775,7 +775,7 @@
     </x:row>
     <x:row r="36" ht="28.5" customHeight="1">
       <x:c r="A36" s="7" t="str">
-        <x:v>Revisión de fuentes públicas: SHA256 4ad6b113996c757d. Sin datos privados.</x:v>
+        <x:v>Revisión de fuentes públicas: SHA256 434cc5a8d9df5142. Sin datos privados.</x:v>
       </x:c>
       <x:c r="B36" s="7"/>
       <x:c r="C36" s="7"/>
@@ -979,10 +979,10 @@
         <x:v>Reunir los escenarios implementados; no implica cubrir todo el ERP.</x:v>
       </x:c>
       <x:c r="E8" s="13" t="n">
-        <x:v>7</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F8" s="13" t="n">
-        <x:v>7</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="13" t="n">
         <x:v>0</x:v>
@@ -1101,10 +1101,10 @@
         <x:v>Cargar productos, cobrar, cancelar y continuar vendiendo.</x:v>
       </x:c>
       <x:c r="E12" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F12" s="13" t="n">
-        <x:v>7</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G12" s="13" t="n">
         <x:v>0</x:v>
@@ -1134,16 +1134,16 @@
         <x:v>Agregar artículos por código o búsqueda y establecer sus cantidades.</x:v>
       </x:c>
       <x:c r="E13" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F13" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G13" s="12" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H13" s="3" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Parcial: ejecutable</x:v>
       </x:c>
       <x:c r="I13" s="3" t="str">
         <x:v>XG-VEN-003, XG-VEN-004</x:v>
@@ -1163,16 +1163,16 @@
         <x:v>Cambiar cantidades, quitar renglones y revisar el total antes de confirmar.</x:v>
       </x:c>
       <x:c r="E14" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F14" s="13" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G14" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H14" s="7" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Parcial: ejecutable</x:v>
       </x:c>
       <x:c r="I14" s="7" t="str">
         <x:v>XG-VEN-003, XG-VEN-007</x:v>
@@ -1192,10 +1192,10 @@
         <x:v>Confirmar el importe recibido, el vuelto y la continuación de la venta.</x:v>
       </x:c>
       <x:c r="E15" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F15" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G15" s="12" t="n">
         <x:v>0</x:v>
@@ -1338,10 +1338,10 @@
         <x:v>Seleccionar medios de pago y verificar importes y cancelaciones del cobro.</x:v>
       </x:c>
       <x:c r="E20" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F20" s="13" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G20" s="13" t="n">
         <x:v>0</x:v>
@@ -1968,7 +1968,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra574c61dd6e14ab3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98215a9e9cdc406d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2348,7 +2348,7 @@
         <x:v>Cargar un producto y modificar su cantidad</x:v>
       </x:c>
       <x:c r="C14" s="7" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D14" s="7" t="str">
         <x:v>Pendiente</x:v>
@@ -2369,11 +2369,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-003.md</x:v>
       </x:c>
-      <x:c r="I14" s="7" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I14" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
       <x:c r="J14" s="7" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="67.5" customHeight="1">
@@ -2384,7 +2385,7 @@
         <x:v>Buscar un código inexistente sin alterar la venta</x:v>
       </x:c>
       <x:c r="C15" s="3" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D15" s="3" t="str">
         <x:v>Pendiente</x:v>
@@ -2404,11 +2405,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-004.md</x:v>
       </x:c>
-      <x:c r="I15" s="3" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I15" s="10" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
       <x:c r="J15" s="3" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="67.5" customHeight="1">
@@ -2419,7 +2421,7 @@
         <x:v>Cobrar en efectivo con vuelto</x:v>
       </x:c>
       <x:c r="C16" s="7" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D16" s="7" t="str">
         <x:v>Pendiente</x:v>
@@ -2439,11 +2441,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-005.md</x:v>
       </x:c>
-      <x:c r="I16" s="7" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I16" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
       <x:c r="J16" s="7" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="67.5" customHeight="1">
@@ -2454,7 +2457,7 @@
         <x:v>Cancelar el cobro, retomarlo y cobrar una sola vez</x:v>
       </x:c>
       <x:c r="C17" s="3" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D17" s="3" t="str">
         <x:v>Pendiente</x:v>
@@ -2475,11 +2478,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-006.md</x:v>
       </x:c>
-      <x:c r="I17" s="3" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I17" s="10" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
       <x:c r="J17" s="3" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="67.5" customHeight="1">
@@ -2490,7 +2494,7 @@
         <x:v>Rechazar el abandono y continuar vendiendo</x:v>
       </x:c>
       <x:c r="C18" s="7" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D18" s="7" t="str">
         <x:v>Pendiente</x:v>
@@ -2510,11 +2514,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-007.md</x:v>
       </x:c>
-      <x:c r="I18" s="7" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I18" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
       <x:c r="J18" s="7" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="67.5" customHeight="1">
@@ -2525,7 +2530,7 @@
         <x:v>Comenzar otra venta después de cobrar</x:v>
       </x:c>
       <x:c r="C19" s="3" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D19" s="3" t="str">
         <x:v>Pendiente</x:v>
@@ -2544,11 +2549,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-008.md</x:v>
       </x:c>
-      <x:c r="I19" s="3" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I19" s="10" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
       <x:c r="J19" s="3" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="67.5" customHeight="1">
@@ -2559,7 +2565,7 @@
         <x:v>Comenzar otra venta después de abandonar</x:v>
       </x:c>
       <x:c r="C20" s="7" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D20" s="7" t="str">
         <x:v>Pendiente</x:v>
@@ -2578,11 +2584,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-009.md</x:v>
       </x:c>
-      <x:c r="I20" s="7" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I20" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
       <x:c r="J20" s="7" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2597,7 +2604,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d1d50b8f5dc4334"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f17b66f993f4cbe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2752,7 +2759,7 @@
         <x:v>Cantidad, código ausente, conservar líneas y continuar.</x:v>
       </x:c>
       <x:c r="E9" s="3" t="str">
-        <x:v>Carga básica incluida en VEN-001/002; variantes VEN-003/004/007 planificadas.</x:v>
+        <x:v>Carga, código ausente y edición incluidos en VEN-001/002/003/004/007; calibración y E2E real pendientes.</x:v>
       </x:c>
       <x:c r="F9" s="3" t="str">
         <x:v>Por detallar / ampliar</x:v>
@@ -2776,7 +2783,7 @@
         <x:v>Exacto, vuelto, cancelar/retomar, abandono y operación siguiente.</x:v>
       </x:c>
       <x:c r="E10" s="7" t="str">
-        <x:v>VEN-001/002 disponibles; VEN-005/006/008/009 planificados.</x:v>
+        <x:v>VEN-001/002/005/006/008/009 disponibles; requieren calibración y ejecución real.</x:v>
       </x:c>
       <x:c r="F10" s="7" t="str">
         <x:v>Por detallar / ampliar</x:v>
@@ -3064,7 +3071,7 @@
         <x:v>Rechazar, cancelar, corregir/reintentar, límites y fallas sin datos parciales/duplicados.</x:v>
       </x:c>
       <x:c r="E22" s="7" t="str">
-        <x:v>Abandono simple disponible; recuperación restante pendiente por familia.</x:v>
+        <x:v>Abandono, rechazo con continuación, edición, cancelar/retomar cobro y siguiente operación disponibles; otras familias pendientes.</x:v>
       </x:c>
       <x:c r="F22" s="7" t="str">
         <x:v>Por detallar / ampliar</x:v>
@@ -3095,7 +3102,7 @@
       </x:c>
       <x:c r="G23" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L56</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L58</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="67.5" customHeight="1">
@@ -3119,7 +3126,7 @@
       </x:c>
       <x:c r="G24" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L57</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L59</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="67.5" customHeight="1">
@@ -3143,7 +3150,7 @@
       </x:c>
       <x:c r="G25" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L58</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L60</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="67.5" customHeight="1">
@@ -3167,7 +3174,7 @@
       </x:c>
       <x:c r="G26" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L59</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L61</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="67.5" customHeight="1">
@@ -3191,7 +3198,7 @@
       </x:c>
       <x:c r="G27" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L60</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L62</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="67.5" customHeight="1">
@@ -3215,7 +3222,7 @@
       </x:c>
       <x:c r="G28" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L61</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L63</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="81" customHeight="1">
@@ -3239,7 +3246,7 @@
       </x:c>
       <x:c r="G29" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L71</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L73</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="67.5" customHeight="1">
@@ -3263,7 +3270,7 @@
       </x:c>
       <x:c r="G30" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L72</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L74</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="67.5" customHeight="1">
@@ -3287,7 +3294,7 @@
       </x:c>
       <x:c r="G31" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L73</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L75</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="67.5" customHeight="1">
@@ -3311,7 +3318,7 @@
       </x:c>
       <x:c r="G32" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L74</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L76</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="67.5" customHeight="1">
@@ -3335,7 +3342,7 @@
       </x:c>
       <x:c r="G33" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L75</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L77</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="67.5" customHeight="1">
@@ -3359,7 +3366,7 @@
       </x:c>
       <x:c r="G34" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L97</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L99</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="67.5" customHeight="1">
@@ -3383,7 +3390,7 @@
       </x:c>
       <x:c r="G35" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L98</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L100</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="67.5" customHeight="1">
@@ -3407,7 +3414,7 @@
       </x:c>
       <x:c r="G36" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L99</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L101</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="67.5" customHeight="1">
@@ -3431,7 +3438,7 @@
       </x:c>
       <x:c r="G37" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L100</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L102</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="67.5" customHeight="1">
@@ -3455,7 +3462,7 @@
       </x:c>
       <x:c r="G38" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L101</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L103</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="67.5" customHeight="1">
@@ -3479,7 +3486,7 @@
       </x:c>
       <x:c r="G39" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L111</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L113</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="67.5" customHeight="1">
@@ -3503,7 +3510,7 @@
       </x:c>
       <x:c r="G40" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L112</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L114</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="67.5" customHeight="1">
@@ -3527,7 +3534,7 @@
       </x:c>
       <x:c r="G41" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L113</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L115</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="67.5" customHeight="1">
@@ -3551,7 +3558,7 @@
       </x:c>
       <x:c r="G42" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L114</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L116</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="67.5" customHeight="1">
@@ -3575,7 +3582,7 @@
       </x:c>
       <x:c r="G43" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L115</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L117</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="67.5" customHeight="1">
@@ -3599,7 +3606,7 @@
       </x:c>
       <x:c r="G44" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L116</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L118</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="67.5" customHeight="1">
@@ -3623,7 +3630,7 @@
       </x:c>
       <x:c r="G45" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L117</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L119</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="67.5" customHeight="1">
@@ -3647,7 +3654,7 @@
       </x:c>
       <x:c r="G46" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L118</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L120</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="67.5" customHeight="1">
@@ -3671,7 +3678,7 @@
       </x:c>
       <x:c r="G47" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L119</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L121</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="67.5" customHeight="1">
@@ -3695,7 +3702,7 @@
       </x:c>
       <x:c r="G48" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L120</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L122</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="67.5" customHeight="1">
@@ -3719,7 +3726,7 @@
       </x:c>
       <x:c r="G49" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L121</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L123</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="67.5" customHeight="1">
@@ -3743,7 +3750,7 @@
       </x:c>
       <x:c r="G50" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L122</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L124</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="67.5" customHeight="1">
@@ -3767,7 +3774,7 @@
       </x:c>
       <x:c r="G51" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L123</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L125</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="67.5" customHeight="1">
@@ -3791,7 +3798,7 @@
       </x:c>
       <x:c r="G52" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L124</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L126</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="67.5" customHeight="1">
@@ -3815,7 +3822,7 @@
       </x:c>
       <x:c r="G53" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L125</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L127</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="67.5" customHeight="1">
@@ -3839,7 +3846,7 @@
       </x:c>
       <x:c r="G54" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L126</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L128</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="67.5" customHeight="1">
@@ -3863,7 +3870,7 @@
       </x:c>
       <x:c r="G55" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L127</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L129</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="67.5" customHeight="1">
@@ -3887,7 +3894,7 @@
       </x:c>
       <x:c r="G56" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L128</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L130</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="67.5" customHeight="1">
@@ -3911,7 +3918,7 @@
       </x:c>
       <x:c r="G57" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L129</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L131</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="67.5" customHeight="1">
@@ -3935,7 +3942,7 @@
       </x:c>
       <x:c r="G58" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L130</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L132</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3944,7 +3951,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R152cfd9fd39d439a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd937c541bf7748bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4871,7 +4878,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a2fbbe6e9834c74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12abfbed683d4aa7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[test] - Incorporar contrato de ventas por teclado
Agrega la ruta JAB para editar renglones de forma segura, conserva el fallback por doble clic hasta validar el FAT JAR y documenta la calibración y el backlog de Restobar.
</commit_message>
<xml_diff>
--- a/docs/coverage/xgestion-cobertura.xlsx
+++ b/docs/coverage/xgestion-cobertura.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R93a9a537d9eb4d92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="2" r:id="R6c55d5c238a74a25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenarios" sheetId="3" r:id="R963b9572bf9a4b8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por detallar" sheetId="4" r:id="Rfbea94cef47a4a5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplos seed" sheetId="5" r:id="R5153ee3f4c0342fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R2fc8931331214cef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="2" r:id="R3808f98b36034a0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenarios" sheetId="3" r:id="Ra0f95cfe51194626"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por detallar" sheetId="4" r:id="R81c784dc184f4904"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplos seed" sheetId="5" r:id="R80267cc998334847"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -775,7 +775,7 @@
     </x:row>
     <x:row r="36" ht="28.5" customHeight="1">
       <x:c r="A36" s="7" t="str">
-        <x:v>Revisión de fuentes públicas: SHA256 434cc5a8d9df5142. Sin datos privados.</x:v>
+        <x:v>Revisión de fuentes públicas: SHA256 4f2143c050118b3a. Sin datos privados.</x:v>
       </x:c>
       <x:c r="B36" s="7"/>
       <x:c r="C36" s="7"/>
@@ -1968,7 +1968,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98215a9e9cdc406d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ca1a129dfa14085"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2604,7 +2604,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f17b66f993f4cbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra25797128bcd449e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3951,7 +3951,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd937c541bf7748bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cc04cfa70054e27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4878,7 +4878,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12abfbed683d4aa7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbc74f6aa1cd4661"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[docs] - Actualiza el backlog de accesibilidad de XGestión
Registra la implementación técnica de XG-ACC-002 a XG-ACC-005, documenta los atajos y la validación pendiente sobre FAT JAR y JAB. Regenera los artefactos de cobertura sin presentar Restobar como parte de los casos ejecutables de Venta.
</commit_message>
<xml_diff>
--- a/docs/coverage/xgestion-cobertura.xlsx
+++ b/docs/coverage/xgestion-cobertura.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R2fc8931331214cef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="2" r:id="R3808f98b36034a0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenarios" sheetId="3" r:id="Ra0f95cfe51194626"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por detallar" sheetId="4" r:id="R81c784dc184f4904"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplos seed" sheetId="5" r:id="R80267cc998334847"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Ra309227d8d714ad3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="2" r:id="R9fd9f7eca346439a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenarios" sheetId="3" r:id="R7e5675f3a47f41c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por detallar" sheetId="4" r:id="Rcab0ffae4afc4623"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplos seed" sheetId="5" r:id="R88be0ea8aafe4945"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -775,7 +775,7 @@
     </x:row>
     <x:row r="36" ht="28.5" customHeight="1">
       <x:c r="A36" s="7" t="str">
-        <x:v>Revisión de fuentes públicas: SHA256 4f2143c050118b3a. Sin datos privados.</x:v>
+        <x:v>Revisión de fuentes públicas: SHA256 cd977255fd8bf407. Sin datos privados.</x:v>
       </x:c>
       <x:c r="B36" s="7"/>
       <x:c r="C36" s="7"/>
@@ -1968,7 +1968,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ca1a129dfa14085"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd42233dd3199461e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2604,7 +2604,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra25797128bcd449e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R331aec967381426d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3951,7 +3951,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cc04cfa70054e27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R845b6c3ac91e40e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4878,7 +4878,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbc74f6aa1cd4661"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2496d3a5835d47bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[feat] - Automatizar promociones simples de XGestión
Agrega siete escenarios con recálculo por cantidad, cancelación y reanudación del cobro y comprobaciones de bruto, descuento, neto, stock y caja. Prepara automáticamente catalogo-comercial-v1 cuando la selección lo requiere y actualiza la documentación y el mapa Excel a 21 casos implementados.

Validación técnica: 519 tests aprobados, 34 omitidos por requisitos del entorno, lint Python y Robot, catálogo, cobertura y dry-run de los 21 casos. La calibración y ejecución real sobre el JAR continúan pendientes del paquete privado.
</commit_message>
<xml_diff>
--- a/docs/coverage/xgestion-cobertura.xlsx
+++ b/docs/coverage/xgestion-cobertura.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Ra309227d8d714ad3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="2" r:id="R9fd9f7eca346439a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenarios" sheetId="3" r:id="R7e5675f3a47f41c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por detallar" sheetId="4" r:id="Rcab0ffae4afc4623"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplos seed" sheetId="5" r:id="R88be0ea8aafe4945"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R999c8f546d5e4041"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="2" r:id="Rb855d9d923f345c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenarios" sheetId="3" r:id="R79ed09ebbf784ee0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por detallar" sheetId="4" r:id="R4a8ae16b61294d3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplos seed" sheetId="5" r:id="Ree66502519d54393"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -210,8 +210,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ScenariosTable" displayName="ScenariosTable" ref="A6:J20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:J20"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ScenariosTable" displayName="ScenariosTable" ref="A6:J27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:J27"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Recorrido del usuario"/>
@@ -245,18 +245,19 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SeedExamplesTable" displayName="SeedExamplesTable" ref="A6:I32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:I32"/>
-  <x:tableColumns count="9">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SeedExamplesTable" displayName="SeedExamplesTable" ref="A6:J32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:J32"/>
+  <x:tableColumns count="10">
     <x:tableColumn id="1" name="Ejemplo"/>
     <x:tableColumn id="2" name="Productos × cantidades"/>
     <x:tableColumn id="3" name="Lista"/>
     <x:tableColumn id="4" name="Total esperado"/>
     <x:tableColumn id="5" name="Moneda"/>
-    <x:tableColumn id="6" name="Estado"/>
-    <x:tableColumn id="7" name="Condiciones"/>
-    <x:tableColumn id="8" name="Datos"/>
-    <x:tableColumn id="9" name="Trazabilidad ERP"/>
+    <x:tableColumn id="6" name="Validación real"/>
+    <x:tableColumn id="7" name="Escenario E2E"/>
+    <x:tableColumn id="8" name="Condiciones"/>
+    <x:tableColumn id="9" name="Datos"/>
+    <x:tableColumn id="10" name="Trazabilidad ERP"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -510,8 +511,8 @@
         <x:v>Documentadas (IDs únicos)</x:v>
       </x:c>
       <x:c r="B7" s="21" t="n">
-        <x:f>COUNTA('Escenarios'!$A$7:$A$20)</x:f>
-        <x:v>14</x:v>
+        <x:f>COUNTA('Escenarios'!$A$7:$A$27)</x:f>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C7" s="3" t="str">
         <x:v>Universo de fichas actuales; no representa todo el ERP.</x:v>
@@ -522,8 +523,8 @@
         <x:v>Automatizadas</x:v>
       </x:c>
       <x:c r="B8" s="21" t="n">
-        <x:f>COUNTIF('Escenarios'!$C$7:$C$20,"Automatizado")</x:f>
-        <x:v>14</x:v>
+        <x:f>COUNTIF('Escenarios'!$C$7:$C$27,"Automatizado")</x:f>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C8" s="3" t="str">
         <x:v>Código de prueba disponible. Ejecución real pendiente.</x:v>
@@ -534,7 +535,7 @@
         <x:v>Pendientes de automatizar</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:f>COUNTIF('Escenarios'!$C$7:$C$20,"Pendiente")</x:f>
+        <x:f>COUNTIF('Escenarios'!$C$7:$C$27,"Pendiente")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
@@ -546,7 +547,7 @@
         <x:v>Manuales</x:v>
       </x:c>
       <x:c r="B10" s="21" t="n">
-        <x:f>COUNTIF('Escenarios'!$C$7:$C$20,"Manual")</x:f>
+        <x:f>COUNTIF('Escenarios'!$C$7:$C$27,"Manual")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C10" s="3" t="str">
@@ -558,7 +559,7 @@
         <x:v>Validadas con evidencia pública</x:v>
       </x:c>
       <x:c r="B11" s="23" t="n">
-        <x:f>COUNTIF('Escenarios'!$D$7:$D$20,"Validado")</x:f>
+        <x:f>COUNTIF('Escenarios'!$D$7:$D$27,"Validado")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C11" s="7" t="str">
@@ -591,7 +592,7 @@
         <x:v>XGestión</x:v>
       </x:c>
       <x:c r="B15" s="12" t="n">
-        <x:v>14</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C15" s="3" t="str">
         <x:v>Primeros escenarios implementados; validación real pendiente.</x:v>
@@ -678,10 +679,10 @@
         <x:v>2. Productos y condiciones comerciales</x:v>
       </x:c>
       <x:c r="B24" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C24" s="3" t="str">
-        <x:v>Sin fichas todavía: ver Por detallar.</x:v>
+        <x:v>0 pendientes · 0 manuales</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
@@ -747,7 +748,7 @@
     </x:row>
     <x:row r="32" ht="28.5" customHeight="1">
       <x:c r="A32" s="7" t="str">
-        <x:v>20 recorridos de Restobar y 26 ejemplos del seed pendientes de ficha/automatización; no se suman al total.</x:v>
+        <x:v>20 recorridos Restobar sin ficha. 26 ejemplos seed: 7 vinculados a fichas y 19 sin ficha. No se suman al total.</x:v>
       </x:c>
       <x:c r="B32" s="7"/>
       <x:c r="C32" s="7"/>
@@ -775,7 +776,7 @@
     </x:row>
     <x:row r="36" ht="28.5" customHeight="1">
       <x:c r="A36" s="7" t="str">
-        <x:v>Revisión de fuentes públicas: SHA256 cd977255fd8bf407. Sin datos privados.</x:v>
+        <x:v>Revisión de fuentes públicas: SHA256 91145c3d34a016da. Sin datos privados.</x:v>
       </x:c>
       <x:c r="B36" s="7"/>
       <x:c r="C36" s="7"/>
@@ -965,7 +966,7 @@
 XG-PRO-002</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="108" customHeight="1">
+    <x:row r="8" ht="162" customHeight="1">
       <x:c r="A8" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -979,7 +980,7 @@
         <x:v>Reunir los escenarios implementados; no implica cubrir todo el ERP.</x:v>
       </x:c>
       <x:c r="E8" s="13" t="n">
-        <x:v>14</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F8" s="13" t="n">
         <x:v>0</x:v>
@@ -992,12 +993,16 @@
       </x:c>
       <x:c r="I8" s="7" t="str">
         <x:v>XG-AUT-001, XG-AUT-002
-XG-INI-001, XG-PRO-001
-XG-PRO-002, XG-VEN-001
-XG-VEN-002, XG-VEN-003
-XG-VEN-004, XG-VEN-005
-XG-VEN-006, XG-VEN-007
-XG-VEN-008, XG-VEN-009</x:v>
+XG-INI-001, XG-PRM-001
+XG-PRM-002, XG-PRM-003
+XG-PRM-004, XG-PRM-005
+XG-PRM-006, XG-PRM-007
+XG-PRO-001, XG-PRO-002
+XG-VEN-001, XG-VEN-002
+XG-VEN-003, XG-VEN-004
+XG-VEN-005, XG-VEN-006
+XG-VEN-007, XG-VEN-008
+XG-VEN-009</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="40.5" customHeight="1">
@@ -1266,7 +1271,7 @@
         <x:v>Por detallar</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="40.5" customHeight="1">
+    <x:row r="18" ht="67.5" customHeight="1">
       <x:c r="A18" s="7" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -1277,10 +1282,10 @@
         <x:v>promociones</x:v>
       </x:c>
       <x:c r="D18" s="7" t="str">
-        <x:v>Aplicar ofertas y combos y recalcularlos al modificar la venta.</x:v>
+        <x:v>Comprobar ofertas, su vigencia y el recálculo al modificar cantidades.</x:v>
       </x:c>
       <x:c r="E18" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F18" s="13" t="n">
         <x:v>0</x:v>
@@ -1289,10 +1294,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H18" s="7" t="str">
-        <x:v>Sin fichas</x:v>
+        <x:v>Parcial: ejecutable</x:v>
       </x:c>
       <x:c r="I18" s="7" t="str">
-        <x:v>Por detallar</x:v>
+        <x:v>XG-PRM-001, XG-PRM-002
+XG-PRM-003, XG-PRM-004
+XG-PRM-005, XG-PRM-006
+XG-PRM-007</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="40.5" customHeight="1">
@@ -1968,7 +1976,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd42233dd3199461e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R947b03668899417f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2198,10 +2206,10 @@
     </x:row>
     <x:row r="10" ht="67.5" customHeight="1">
       <x:c r="A10" s="7" t="str">
-        <x:v>XG-PRO-001</x:v>
+        <x:v>XG-PRM-001</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>Buscar producto conocido</x:v>
+        <x:v>Aplicar una promoción porcentual y recalcular la cantidad</x:v>
       </x:c>
       <x:c r="C10" s="7" t="str">
         <x:v>Automatizado</x:v>
@@ -2210,385 +2218,630 @@
         <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="E10" s="7" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F10" s="7" t="str">
+        <x:v>P1/P0</x:v>
+      </x:c>
+      <x:c r="G10" s="7" t="str">
+        <x:v>Regresión disponible [regression]
+Promociones [promociones]</x:v>
+      </x:c>
+      <x:c r="H10" s="11" t="str">
+        <x:v>Ver ficha
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/promociones/XG-PRM-001.md</x:v>
+      </x:c>
+      <x:c r="I10" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/promociones.robot</x:v>
+      </x:c>
+      <x:c r="J10" s="7" t="str">
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="67.5" customHeight="1">
+      <x:c r="A11" s="3" t="str">
+        <x:v>XG-PRM-002</x:v>
+      </x:c>
+      <x:c r="B11" s="3" t="str">
+        <x:v>Aplicar un descuento de importe fijo y recalcular la cantidad</x:v>
+      </x:c>
+      <x:c r="C11" s="3" t="str">
+        <x:v>Automatizado</x:v>
+      </x:c>
+      <x:c r="D11" s="3" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="E11" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F11" s="3" t="str">
+        <x:v>P1/P0</x:v>
+      </x:c>
+      <x:c r="G11" s="3" t="str">
+        <x:v>Regresión disponible [regression]
+Promociones [promociones]</x:v>
+      </x:c>
+      <x:c r="H11" s="10" t="str">
+        <x:v>Ver ficha
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/promociones/XG-PRM-002.md</x:v>
+      </x:c>
+      <x:c r="I11" s="10" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/promociones.robot</x:v>
+      </x:c>
+      <x:c r="J11" s="3" t="str">
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="67.5" customHeight="1">
+      <x:c r="A12" s="7" t="str">
+        <x:v>XG-PRM-003</x:v>
+      </x:c>
+      <x:c r="B12" s="7" t="str">
+        <x:v>Recalcular una promoción 2x1 al pasar de una a tres unidades</x:v>
+      </x:c>
+      <x:c r="C12" s="7" t="str">
+        <x:v>Automatizado</x:v>
+      </x:c>
+      <x:c r="D12" s="7" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="E12" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F12" s="7" t="str">
+        <x:v>P1/P0</x:v>
+      </x:c>
+      <x:c r="G12" s="7" t="str">
+        <x:v>Regresión disponible [regression]
+Promociones [promociones]</x:v>
+      </x:c>
+      <x:c r="H12" s="11" t="str">
+        <x:v>Ver ficha
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/promociones/XG-PRM-003.md</x:v>
+      </x:c>
+      <x:c r="I12" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/promociones.robot</x:v>
+      </x:c>
+      <x:c r="J12" s="7" t="str">
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="67.5" customHeight="1">
+      <x:c r="A13" s="3" t="str">
+        <x:v>XG-PRM-004</x:v>
+      </x:c>
+      <x:c r="B13" s="3" t="str">
+        <x:v>Recalcular el descuento del 50 % en la segunda unidad</x:v>
+      </x:c>
+      <x:c r="C13" s="3" t="str">
+        <x:v>Automatizado</x:v>
+      </x:c>
+      <x:c r="D13" s="3" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="E13" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F13" s="3" t="str">
+        <x:v>P1/P0</x:v>
+      </x:c>
+      <x:c r="G13" s="3" t="str">
+        <x:v>Regresión disponible [regression]
+Promociones [promociones]</x:v>
+      </x:c>
+      <x:c r="H13" s="10" t="str">
+        <x:v>Ver ficha
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/promociones/XG-PRM-004.md</x:v>
+      </x:c>
+      <x:c r="I13" s="10" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/promociones.robot</x:v>
+      </x:c>
+      <x:c r="J13" s="3" t="str">
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="67.5" customHeight="1">
+      <x:c r="A14" s="7" t="str">
+        <x:v>XG-PRM-005</x:v>
+      </x:c>
+      <x:c r="B14" s="7" t="str">
+        <x:v>Conservar el precio normal cuando la promoción está vencida</x:v>
+      </x:c>
+      <x:c r="C14" s="7" t="str">
+        <x:v>Automatizado</x:v>
+      </x:c>
+      <x:c r="D14" s="7" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="E14" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F14" s="7" t="str">
+        <x:v>P1/P0</x:v>
+      </x:c>
+      <x:c r="G14" s="7" t="str">
+        <x:v>Regresión disponible [regression]
+Promociones [promociones]</x:v>
+      </x:c>
+      <x:c r="H14" s="11" t="str">
+        <x:v>Ver ficha
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/promociones/XG-PRM-005.md</x:v>
+      </x:c>
+      <x:c r="I14" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/promociones.robot</x:v>
+      </x:c>
+      <x:c r="J14" s="7" t="str">
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="67.5" customHeight="1">
+      <x:c r="A15" s="3" t="str">
+        <x:v>XG-PRM-006</x:v>
+      </x:c>
+      <x:c r="B15" s="3" t="str">
+        <x:v>Conservar el precio normal antes del inicio de una promoción</x:v>
+      </x:c>
+      <x:c r="C15" s="3" t="str">
+        <x:v>Automatizado</x:v>
+      </x:c>
+      <x:c r="D15" s="3" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="E15" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F15" s="3" t="str">
+        <x:v>P1/P0</x:v>
+      </x:c>
+      <x:c r="G15" s="3" t="str">
+        <x:v>Regresión disponible [regression]
+Promociones [promociones]</x:v>
+      </x:c>
+      <x:c r="H15" s="10" t="str">
+        <x:v>Ver ficha
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/promociones/XG-PRM-006.md</x:v>
+      </x:c>
+      <x:c r="I15" s="10" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/promociones.robot</x:v>
+      </x:c>
+      <x:c r="J15" s="3" t="str">
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="67.5" customHeight="1">
+      <x:c r="A16" s="7" t="str">
+        <x:v>XG-PRM-007</x:v>
+      </x:c>
+      <x:c r="B16" s="7" t="str">
+        <x:v>Conservar el precio normal cuando la promoción está desactivada</x:v>
+      </x:c>
+      <x:c r="C16" s="7" t="str">
+        <x:v>Automatizado</x:v>
+      </x:c>
+      <x:c r="D16" s="7" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="E16" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F16" s="7" t="str">
+        <x:v>P1/P0</x:v>
+      </x:c>
+      <x:c r="G16" s="7" t="str">
+        <x:v>Regresión disponible [regression]
+Promociones [promociones]</x:v>
+      </x:c>
+      <x:c r="H16" s="11" t="str">
+        <x:v>Ver ficha
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/promociones/XG-PRM-007.md</x:v>
+      </x:c>
+      <x:c r="I16" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/promociones.robot</x:v>
+      </x:c>
+      <x:c r="J16" s="7" t="str">
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="67.5" customHeight="1">
+      <x:c r="A17" s="3" t="str">
+        <x:v>XG-PRO-001</x:v>
+      </x:c>
+      <x:c r="B17" s="3" t="str">
+        <x:v>Buscar producto conocido</x:v>
+      </x:c>
+      <x:c r="C17" s="3" t="str">
+        <x:v>Automatizado</x:v>
+      </x:c>
+      <x:c r="D17" s="3" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="E17" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F17" s="3" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G10" s="7" t="str">
+      <x:c r="G17" s="3" t="str">
         <x:v>Comprobación rápida [smoke]
 Regresión disponible [regression]
 Búsqueda de productos [productos]</x:v>
       </x:c>
-      <x:c r="H10" s="11" t="str">
+      <x:c r="H17" s="10" t="str">
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/productos/XG-PRO-001.md</x:v>
       </x:c>
-      <x:c r="I10" s="11" t="str">
+      <x:c r="I17" s="10" t="str">
         <x:v>Ver prueba
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/smoke.robot</x:v>
       </x:c>
-      <x:c r="J10" s="7" t="str">
+      <x:c r="J17" s="3" t="str">
         <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="67.5" customHeight="1">
-      <x:c r="A11" s="3" t="str">
+    <x:row r="18" ht="67.5" customHeight="1">
+      <x:c r="A18" s="7" t="str">
         <x:v>XG-PRO-002</x:v>
       </x:c>
-      <x:c r="B11" s="3" t="str">
+      <x:c r="B18" s="7" t="str">
         <x:v>Buscar producto inexistente</x:v>
       </x:c>
-      <x:c r="C11" s="3" t="str">
+      <x:c r="C18" s="7" t="str">
         <x:v>Automatizado</x:v>
       </x:c>
-      <x:c r="D11" s="3" t="str">
+      <x:c r="D18" s="7" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
-      <x:c r="E11" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F11" s="3" t="str">
+      <x:c r="E18" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F18" s="7" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G11" s="3" t="str">
+      <x:c r="G18" s="7" t="str">
         <x:v>Comprobación rápida [smoke]
 Regresión disponible [regression]
 Búsqueda de productos [productos]</x:v>
       </x:c>
-      <x:c r="H11" s="10" t="str">
+      <x:c r="H18" s="11" t="str">
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/productos/XG-PRO-002.md</x:v>
       </x:c>
-      <x:c r="I11" s="10" t="str">
+      <x:c r="I18" s="11" t="str">
         <x:v>Ver prueba
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/smoke.robot</x:v>
       </x:c>
-      <x:c r="J11" s="3" t="str">
+      <x:c r="J18" s="7" t="str">
         <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="67.5" customHeight="1">
-      <x:c r="A12" s="7" t="str">
+    <x:row r="19" ht="67.5" customHeight="1">
+      <x:c r="A19" s="3" t="str">
         <x:v>XG-VEN-001</x:v>
       </x:c>
-      <x:c r="B12" s="7" t="str">
+      <x:c r="B19" s="3" t="str">
         <x:v>Venta no fiscal en efectivo</x:v>
       </x:c>
-      <x:c r="C12" s="7" t="str">
+      <x:c r="C19" s="3" t="str">
         <x:v>Automatizado</x:v>
       </x:c>
-      <x:c r="D12" s="7" t="str">
+      <x:c r="D19" s="3" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
-      <x:c r="E12" s="7" t="n">
+      <x:c r="E19" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F12" s="7" t="str">
+      <x:c r="F19" s="3" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G12" s="7" t="str">
+      <x:c r="G19" s="3" t="str">
         <x:v>Regresión disponible [regression]
 Venta cotidiana [ventas]
 Cobrar en efectivo [efectivo]
 Formas de cobro [cobros]</x:v>
       </x:c>
-      <x:c r="H12" s="11" t="str">
+      <x:c r="H19" s="10" t="str">
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-001.md</x:v>
       </x:c>
-      <x:c r="I12" s="11" t="str">
+      <x:c r="I19" s="10" t="str">
         <x:v>Ver prueba
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
-      <x:c r="J12" s="7" t="str">
+      <x:c r="J19" s="3" t="str">
         <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="67.5" customHeight="1">
-      <x:c r="A13" s="3" t="str">
+    <x:row r="20" ht="67.5" customHeight="1">
+      <x:c r="A20" s="7" t="str">
         <x:v>XG-VEN-002</x:v>
       </x:c>
-      <x:c r="B13" s="3" t="str">
+      <x:c r="B20" s="7" t="str">
         <x:v>Cancelar venta sin persistir</x:v>
       </x:c>
-      <x:c r="C13" s="3" t="str">
+      <x:c r="C20" s="7" t="str">
         <x:v>Automatizado</x:v>
       </x:c>
-      <x:c r="D13" s="3" t="str">
+      <x:c r="D20" s="7" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
-      <x:c r="E13" s="3" t="n">
+      <x:c r="E20" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F13" s="3" t="str">
+      <x:c r="F20" s="7" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G13" s="3" t="str">
+      <x:c r="G20" s="7" t="str">
         <x:v>Regresión disponible [regression]
 Venta cotidiana [ventas]</x:v>
       </x:c>
-      <x:c r="H13" s="10" t="str">
+      <x:c r="H20" s="11" t="str">
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-002.md</x:v>
       </x:c>
-      <x:c r="I13" s="10" t="str">
+      <x:c r="I20" s="11" t="str">
         <x:v>Ver prueba
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
-      <x:c r="J13" s="3" t="str">
+      <x:c r="J20" s="7" t="str">
         <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="81" customHeight="1">
-      <x:c r="A14" s="7" t="str">
+    <x:row r="21" ht="81" customHeight="1">
+      <x:c r="A21" s="3" t="str">
         <x:v>XG-VEN-003</x:v>
       </x:c>
-      <x:c r="B14" s="7" t="str">
+      <x:c r="B21" s="3" t="str">
         <x:v>Cargar un producto y modificar su cantidad</x:v>
       </x:c>
-      <x:c r="C14" s="7" t="str">
+      <x:c r="C21" s="3" t="str">
         <x:v>Automatizado</x:v>
       </x:c>
-      <x:c r="D14" s="7" t="str">
+      <x:c r="D21" s="3" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
-      <x:c r="E14" s="7" t="n">
+      <x:c r="E21" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F14" s="7" t="str">
+      <x:c r="F21" s="3" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G14" s="7" t="str">
+      <x:c r="G21" s="3" t="str">
         <x:v>Regresión disponible [regression]
 Venta cotidiana [ventas]
 Cargar productos en la venta [carga-productos]
 Corregir una venta [corregir-venta]</x:v>
       </x:c>
-      <x:c r="H14" s="11" t="str">
+      <x:c r="H21" s="10" t="str">
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-003.md</x:v>
       </x:c>
-      <x:c r="I14" s="11" t="str">
+      <x:c r="I21" s="10" t="str">
         <x:v>Ver prueba
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
-      <x:c r="J14" s="7" t="str">
+      <x:c r="J21" s="3" t="str">
         <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="67.5" customHeight="1">
-      <x:c r="A15" s="3" t="str">
+    <x:row r="22" ht="67.5" customHeight="1">
+      <x:c r="A22" s="7" t="str">
         <x:v>XG-VEN-004</x:v>
       </x:c>
-      <x:c r="B15" s="3" t="str">
+      <x:c r="B22" s="7" t="str">
         <x:v>Buscar un código inexistente sin alterar la venta</x:v>
       </x:c>
-      <x:c r="C15" s="3" t="str">
+      <x:c r="C22" s="7" t="str">
         <x:v>Automatizado</x:v>
       </x:c>
-      <x:c r="D15" s="3" t="str">
+      <x:c r="D22" s="7" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
-      <x:c r="E15" s="3" t="n">
+      <x:c r="E22" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F15" s="3" t="str">
+      <x:c r="F22" s="7" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G15" s="3" t="str">
+      <x:c r="G22" s="7" t="str">
         <x:v>Regresión disponible [regression]
 Venta cotidiana [ventas]
 Cargar productos en la venta [carga-productos]</x:v>
       </x:c>
-      <x:c r="H15" s="10" t="str">
+      <x:c r="H22" s="11" t="str">
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-004.md</x:v>
       </x:c>
-      <x:c r="I15" s="10" t="str">
+      <x:c r="I22" s="11" t="str">
         <x:v>Ver prueba
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
-      <x:c r="J15" s="3" t="str">
+      <x:c r="J22" s="7" t="str">
         <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="67.5" customHeight="1">
-      <x:c r="A16" s="7" t="str">
+    <x:row r="23" ht="67.5" customHeight="1">
+      <x:c r="A23" s="3" t="str">
         <x:v>XG-VEN-005</x:v>
       </x:c>
-      <x:c r="B16" s="7" t="str">
+      <x:c r="B23" s="3" t="str">
         <x:v>Cobrar en efectivo con vuelto</x:v>
       </x:c>
-      <x:c r="C16" s="7" t="str">
+      <x:c r="C23" s="3" t="str">
         <x:v>Automatizado</x:v>
       </x:c>
-      <x:c r="D16" s="7" t="str">
+      <x:c r="D23" s="3" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
-      <x:c r="E16" s="7" t="n">
+      <x:c r="E23" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F16" s="7" t="str">
+      <x:c r="F23" s="3" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G16" s="7" t="str">
+      <x:c r="G23" s="3" t="str">
         <x:v>Regresión disponible [regression]
 Venta cotidiana [ventas]
 Cobrar en efectivo [efectivo]</x:v>
       </x:c>
-      <x:c r="H16" s="11" t="str">
+      <x:c r="H23" s="10" t="str">
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-005.md</x:v>
       </x:c>
-      <x:c r="I16" s="11" t="str">
+      <x:c r="I23" s="10" t="str">
         <x:v>Ver prueba
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
-      <x:c r="J16" s="7" t="str">
+      <x:c r="J23" s="3" t="str">
         <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="67.5" customHeight="1">
-      <x:c r="A17" s="3" t="str">
+    <x:row r="24" ht="67.5" customHeight="1">
+      <x:c r="A24" s="7" t="str">
         <x:v>XG-VEN-006</x:v>
       </x:c>
-      <x:c r="B17" s="3" t="str">
+      <x:c r="B24" s="7" t="str">
         <x:v>Cancelar el cobro, retomarlo y cobrar una sola vez</x:v>
       </x:c>
-      <x:c r="C17" s="3" t="str">
+      <x:c r="C24" s="7" t="str">
         <x:v>Automatizado</x:v>
       </x:c>
-      <x:c r="D17" s="3" t="str">
+      <x:c r="D24" s="7" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
-      <x:c r="E17" s="3" t="n">
+      <x:c r="E24" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F17" s="3" t="str">
+      <x:c r="F24" s="7" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G17" s="3" t="str">
+      <x:c r="G24" s="7" t="str">
         <x:v>Regresión disponible [regression]
 Venta cotidiana [ventas]
 Cobrar en efectivo [efectivo]
 Formas de cobro [cobros]</x:v>
       </x:c>
-      <x:c r="H17" s="10" t="str">
+      <x:c r="H24" s="11" t="str">
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-006.md</x:v>
       </x:c>
-      <x:c r="I17" s="10" t="str">
+      <x:c r="I24" s="11" t="str">
         <x:v>Ver prueba
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
-      <x:c r="J17" s="3" t="str">
+      <x:c r="J24" s="7" t="str">
         <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="67.5" customHeight="1">
-      <x:c r="A18" s="7" t="str">
+    <x:row r="25" ht="67.5" customHeight="1">
+      <x:c r="A25" s="3" t="str">
         <x:v>XG-VEN-007</x:v>
       </x:c>
-      <x:c r="B18" s="7" t="str">
+      <x:c r="B25" s="3" t="str">
         <x:v>Rechazar el abandono y continuar vendiendo</x:v>
       </x:c>
-      <x:c r="C18" s="7" t="str">
+      <x:c r="C25" s="3" t="str">
         <x:v>Automatizado</x:v>
       </x:c>
-      <x:c r="D18" s="7" t="str">
+      <x:c r="D25" s="3" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
-      <x:c r="E18" s="7" t="n">
+      <x:c r="E25" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F18" s="7" t="str">
+      <x:c r="F25" s="3" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G18" s="7" t="str">
+      <x:c r="G25" s="3" t="str">
         <x:v>Regresión disponible [regression]
 Venta cotidiana [ventas]
 Corregir una venta [corregir-venta]</x:v>
       </x:c>
-      <x:c r="H18" s="11" t="str">
+      <x:c r="H25" s="10" t="str">
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-007.md</x:v>
       </x:c>
-      <x:c r="I18" s="11" t="str">
+      <x:c r="I25" s="10" t="str">
         <x:v>Ver prueba
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
-      <x:c r="J18" s="7" t="str">
+      <x:c r="J25" s="3" t="str">
         <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="67.5" customHeight="1">
-      <x:c r="A19" s="3" t="str">
+    <x:row r="26" ht="67.5" customHeight="1">
+      <x:c r="A26" s="7" t="str">
         <x:v>XG-VEN-008</x:v>
       </x:c>
-      <x:c r="B19" s="3" t="str">
+      <x:c r="B26" s="7" t="str">
         <x:v>Comenzar otra venta después de cobrar</x:v>
       </x:c>
-      <x:c r="C19" s="3" t="str">
+      <x:c r="C26" s="7" t="str">
         <x:v>Automatizado</x:v>
       </x:c>
-      <x:c r="D19" s="3" t="str">
+      <x:c r="D26" s="7" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
-      <x:c r="E19" s="3" t="n">
+      <x:c r="E26" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F19" s="3" t="str">
+      <x:c r="F26" s="7" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G19" s="3" t="str">
+      <x:c r="G26" s="7" t="str">
         <x:v>Regresión disponible [regression]
 Venta cotidiana [ventas]</x:v>
       </x:c>
-      <x:c r="H19" s="10" t="str">
+      <x:c r="H26" s="11" t="str">
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-008.md</x:v>
       </x:c>
-      <x:c r="I19" s="10" t="str">
+      <x:c r="I26" s="11" t="str">
         <x:v>Ver prueba
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
-      <x:c r="J19" s="3" t="str">
+      <x:c r="J26" s="7" t="str">
         <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="67.5" customHeight="1">
-      <x:c r="A20" s="7" t="str">
+    <x:row r="27" ht="67.5" customHeight="1">
+      <x:c r="A27" s="3" t="str">
         <x:v>XG-VEN-009</x:v>
       </x:c>
-      <x:c r="B20" s="7" t="str">
+      <x:c r="B27" s="3" t="str">
         <x:v>Comenzar otra venta después de abandonar</x:v>
       </x:c>
-      <x:c r="C20" s="7" t="str">
+      <x:c r="C27" s="3" t="str">
         <x:v>Automatizado</x:v>
       </x:c>
-      <x:c r="D20" s="7" t="str">
+      <x:c r="D27" s="3" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
-      <x:c r="E20" s="7" t="n">
+      <x:c r="E27" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F20" s="7" t="str">
+      <x:c r="F27" s="3" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G20" s="7" t="str">
+      <x:c r="G27" s="3" t="str">
         <x:v>Regresión disponible [regression]
 Venta cotidiana [ventas]</x:v>
       </x:c>
-      <x:c r="H20" s="11" t="str">
+      <x:c r="H27" s="10" t="str">
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/ventas/XG-VEN-009.md</x:v>
       </x:c>
-      <x:c r="I20" s="11" t="str">
+      <x:c r="I27" s="10" t="str">
         <x:v>Ver prueba
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/ventas.robot</x:v>
       </x:c>
-      <x:c r="J20" s="7" t="str">
+      <x:c r="J27" s="3" t="str">
         <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
@@ -2596,15 +2849,15 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:J4"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="C7:C20">
+  <x:conditionalFormatting sqref="C7:C27">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Automatizado"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="C7:D20">
+  <x:conditionalFormatting sqref="C7:D27">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Pendiente"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R331aec967381426d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47c28ab41aef4c19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2718,7 +2971,7 @@
       </x:c>
       <x:c r="G7" s="10" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L49</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L59</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="67.5" customHeight="1">
@@ -2742,7 +2995,7 @@
       </x:c>
       <x:c r="G8" s="11" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L50</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L60</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="67.5" customHeight="1">
@@ -2766,7 +3019,7 @@
       </x:c>
       <x:c r="G9" s="10" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L51</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L61</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="67.5" customHeight="1">
@@ -2790,7 +3043,7 @@
       </x:c>
       <x:c r="G10" s="11" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L52</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L62</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="67.5" customHeight="1">
@@ -2814,10 +3067,10 @@
       </x:c>
       <x:c r="G11" s="10" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L53</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="67.5" customHeight="1">
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L63</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="81" customHeight="1">
       <x:c r="A12" s="7" t="str">
         <x:v>Mapa funcional</x:v>
       </x:c>
@@ -2831,14 +3084,14 @@
         <x:v>Listas por cliente/sucursal/turno/cantidad, porcentaje/importe/cantidad/combos, vigencia y aplicabilidad.</x:v>
       </x:c>
       <x:c r="E12" s="7" t="str">
-        <x:v>Pendiente de fichas y perfiles.</x:v>
+        <x:v>Parcial: PRM-001..007 para porcentaje, importe, 2x1, segunda al 50 % y vencida/futura/inactiva, con edición y cancelación/reintento. Calibración y E2E real pendientes; listas, combos, otros alcances y combinaciones aún sin fichas.</x:v>
       </x:c>
       <x:c r="F12" s="7" t="str">
         <x:v>Por detallar / ampliar</x:v>
       </x:c>
       <x:c r="G12" s="11" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L54</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L64</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="67.5" customHeight="1">
@@ -2862,7 +3115,7 @@
       </x:c>
       <x:c r="G13" s="10" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L55</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L65</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="67.5" customHeight="1">
@@ -2886,7 +3139,7 @@
       </x:c>
       <x:c r="G14" s="11" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L56</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L66</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="67.5" customHeight="1">
@@ -2910,7 +3163,7 @@
       </x:c>
       <x:c r="G15" s="10" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L57</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L67</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="67.5" customHeight="1">
@@ -2934,7 +3187,7 @@
       </x:c>
       <x:c r="G16" s="11" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L58</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L68</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="67.5" customHeight="1">
@@ -2958,7 +3211,7 @@
       </x:c>
       <x:c r="G17" s="10" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L59</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L69</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="67.5" customHeight="1">
@@ -2982,7 +3235,7 @@
       </x:c>
       <x:c r="G18" s="11" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L60</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L70</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="67.5" customHeight="1">
@@ -3006,7 +3259,7 @@
       </x:c>
       <x:c r="G19" s="10" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L61</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L71</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="67.5" customHeight="1">
@@ -3030,7 +3283,7 @@
       </x:c>
       <x:c r="G20" s="11" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L62</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L72</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="67.5" customHeight="1">
@@ -3054,7 +3307,7 @@
       </x:c>
       <x:c r="G21" s="10" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L63</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L73</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="67.5" customHeight="1">
@@ -3071,14 +3324,14 @@
         <x:v>Rechazar, cancelar, corregir/reintentar, límites y fallas sin datos parciales/duplicados.</x:v>
       </x:c>
       <x:c r="E22" s="7" t="str">
-        <x:v>Abandono, rechazo con continuación, edición, cancelar/retomar cobro y siguiente operación disponibles; otras familias pendientes.</x:v>
+        <x:v>Abandono, rechazo con continuación, edición, cancelar/retomar cobro (también en promociones) y siguiente operación disponibles; otras familias pendientes.</x:v>
       </x:c>
       <x:c r="F22" s="7" t="str">
         <x:v>Por detallar / ampliar</x:v>
       </x:c>
       <x:c r="G22" s="11" t="str">
         <x:v>Ver matriz
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L64</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/cobertura.md#L74</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="67.5" customHeight="1">
@@ -3102,7 +3355,7 @@
       </x:c>
       <x:c r="G23" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L58</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L70</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="67.5" customHeight="1">
@@ -3126,7 +3379,7 @@
       </x:c>
       <x:c r="G24" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L59</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L71</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="67.5" customHeight="1">
@@ -3150,7 +3403,7 @@
       </x:c>
       <x:c r="G25" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L60</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L72</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="67.5" customHeight="1">
@@ -3164,17 +3417,17 @@
         <x:v>Ofertas</x:v>
       </x:c>
       <x:c r="D26" s="7" t="str">
-        <x:v>Porcentaje, importe, cantidad y combos; vigencia/aplicabilidad; descuento de ítem/global, cambio de cliente y líneas con notas diferentes.</x:v>
+        <x:v>Primer lote PRM-001..007: porcentaje, importe fijo, 2x1, segunda unidad al 50 %, vencida/futura/inactiva; pendientes combos, demás cantidades/alcances, descuento de ítem/global, cambio de cliente y líneas con notas diferentes.</x:v>
       </x:c>
       <x:c r="E26" s="7" t="str">
-        <x:v>P1/P0 · Recalcular una vez; no perder notas, duplicar beneficios ni superar la base permitida.</x:v>
+        <x:v>P1/P0 · Recalcular una vez; cancelar/retomar sin duplicar beneficios ni cobros. Implementación parcial; validación real y demás combinaciones pendientes.</x:v>
       </x:c>
       <x:c r="F26" s="7" t="str">
         <x:v>Por detallar</x:v>
       </x:c>
       <x:c r="G26" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L61</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L73</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="67.5" customHeight="1">
@@ -3198,7 +3451,7 @@
       </x:c>
       <x:c r="G27" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L62</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L74</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="67.5" customHeight="1">
@@ -3222,7 +3475,7 @@
       </x:c>
       <x:c r="G28" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L63</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L75</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="81" customHeight="1">
@@ -3246,7 +3499,7 @@
       </x:c>
       <x:c r="G29" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L73</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L85</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="67.5" customHeight="1">
@@ -3270,7 +3523,7 @@
       </x:c>
       <x:c r="G30" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L74</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L86</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="67.5" customHeight="1">
@@ -3294,7 +3547,7 @@
       </x:c>
       <x:c r="G31" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L75</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L87</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="67.5" customHeight="1">
@@ -3318,7 +3571,7 @@
       </x:c>
       <x:c r="G32" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L76</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L88</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="67.5" customHeight="1">
@@ -3342,7 +3595,7 @@
       </x:c>
       <x:c r="G33" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L77</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L89</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="67.5" customHeight="1">
@@ -3366,7 +3619,7 @@
       </x:c>
       <x:c r="G34" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L99</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L111</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="67.5" customHeight="1">
@@ -3390,7 +3643,7 @@
       </x:c>
       <x:c r="G35" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L100</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L112</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="67.5" customHeight="1">
@@ -3414,7 +3667,7 @@
       </x:c>
       <x:c r="G36" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L101</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L113</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="67.5" customHeight="1">
@@ -3438,7 +3691,7 @@
       </x:c>
       <x:c r="G37" s="10" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L102</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L114</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="67.5" customHeight="1">
@@ -3462,7 +3715,7 @@
       </x:c>
       <x:c r="G38" s="11" t="str">
         <x:v>Ver roadmap
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L103</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L115</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="67.5" customHeight="1">
@@ -3486,7 +3739,7 @@
       </x:c>
       <x:c r="G39" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L113</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L125</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="67.5" customHeight="1">
@@ -3510,7 +3763,7 @@
       </x:c>
       <x:c r="G40" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L114</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L126</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="67.5" customHeight="1">
@@ -3534,7 +3787,7 @@
       </x:c>
       <x:c r="G41" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L115</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L127</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="67.5" customHeight="1">
@@ -3558,7 +3811,7 @@
       </x:c>
       <x:c r="G42" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L116</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L128</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="67.5" customHeight="1">
@@ -3582,7 +3835,7 @@
       </x:c>
       <x:c r="G43" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L117</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L129</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="67.5" customHeight="1">
@@ -3606,7 +3859,7 @@
       </x:c>
       <x:c r="G44" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L118</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L130</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="67.5" customHeight="1">
@@ -3630,7 +3883,7 @@
       </x:c>
       <x:c r="G45" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L119</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L131</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="67.5" customHeight="1">
@@ -3654,7 +3907,7 @@
       </x:c>
       <x:c r="G46" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L120</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L132</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="67.5" customHeight="1">
@@ -3678,7 +3931,7 @@
       </x:c>
       <x:c r="G47" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L121</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L133</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="67.5" customHeight="1">
@@ -3702,7 +3955,7 @@
       </x:c>
       <x:c r="G48" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L122</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L134</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="67.5" customHeight="1">
@@ -3726,7 +3979,7 @@
       </x:c>
       <x:c r="G49" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L123</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L135</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="67.5" customHeight="1">
@@ -3750,7 +4003,7 @@
       </x:c>
       <x:c r="G50" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L124</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L136</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="67.5" customHeight="1">
@@ -3774,7 +4027,7 @@
       </x:c>
       <x:c r="G51" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L125</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L137</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="67.5" customHeight="1">
@@ -3798,7 +4051,7 @@
       </x:c>
       <x:c r="G52" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L126</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L138</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="67.5" customHeight="1">
@@ -3822,7 +4075,7 @@
       </x:c>
       <x:c r="G53" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L127</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L139</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="67.5" customHeight="1">
@@ -3846,7 +4099,7 @@
       </x:c>
       <x:c r="G54" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L128</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L140</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="67.5" customHeight="1">
@@ -3870,7 +4123,7 @@
       </x:c>
       <x:c r="G55" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L129</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L141</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="67.5" customHeight="1">
@@ -3894,7 +4147,7 @@
       </x:c>
       <x:c r="G56" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L130</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L142</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="67.5" customHeight="1">
@@ -3918,7 +4171,7 @@
       </x:c>
       <x:c r="G57" s="10" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L131</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L143</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="67.5" customHeight="1">
@@ -3942,7 +4195,7 @@
       </x:c>
       <x:c r="G58" s="11" t="str">
         <x:v>Ver recorrido
-https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L132</x:v>
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/docs/roadmap.md#L144</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3951,7 +4204,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R845b6c3ac91e40e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re29031b512dd48f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3968,10 +4221,11 @@
     <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="15.630000114440918" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="9.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="31.25" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="52.5" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="42.5" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="55" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="42.5" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="52.5" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="42.5" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="55" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -3986,6 +4240,7 @@
       <x:c r="G1" s="4"/>
       <x:c r="H1" s="4"/>
       <x:c r="I1" s="4"/>
+      <x:c r="J1" s="4"/>
     </x:row>
     <x:row r="2" ht="6" customHeight="1">
       <x:c r="A2" s="4"/>
@@ -3997,10 +4252,11 @@
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="4"/>
       <x:c r="I2" s="4"/>
+      <x:c r="J2" s="4"/>
     </x:row>
     <x:row r="3" ht="18" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>Datos y resultados esperados para preparar nuevas pruebas. Ninguno de estos ejemplos acredita un E2E. Importes en la moneda indicada; revisar el perfil y las condiciones de la ficha futura.</x:v>
+        <x:v>Datos y resultados esperados. Los ejemplos vinculados tienen su estado de automatización en Escenario E2E. La validación real sigue pendiente; revisar el perfil y las condiciones de cada ficha.</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>
@@ -4010,6 +4266,7 @@
       <x:c r="G3" s="7"/>
       <x:c r="H3" s="7"/>
       <x:c r="I3" s="7"/>
+      <x:c r="J3" s="7"/>
     </x:row>
     <x:row r="4" ht="18" customHeight="1">
       <x:c r="A4" s="7"/>
@@ -4021,6 +4278,7 @@
       <x:c r="G4" s="7"/>
       <x:c r="H4" s="7"/>
       <x:c r="I4" s="7"/>
+      <x:c r="J4" s="7"/>
     </x:row>
     <x:row r="5" ht="10.5" customHeight="1">
       <x:c r="A5" s="3"/>
@@ -4032,6 +4290,7 @@
       <x:c r="G5" s="3"/>
       <x:c r="H5" s="3"/>
       <x:c r="I5" s="3"/>
+      <x:c r="J5" s="3"/>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="9" t="str">
@@ -4050,15 +4309,18 @@
         <x:v>Moneda</x:v>
       </x:c>
       <x:c r="F6" s="9" t="str">
-        <x:v>Estado</x:v>
+        <x:v>Validación real</x:v>
       </x:c>
       <x:c r="G6" s="9" t="str">
+        <x:v>Escenario E2E</x:v>
+      </x:c>
+      <x:c r="H6" s="9" t="str">
         <x:v>Condiciones</x:v>
       </x:c>
-      <x:c r="H6" s="9" t="str">
+      <x:c r="I6" s="9" t="str">
         <x:v>Datos</x:v>
       </x:c>
-      <x:c r="I6" s="9" t="str">
+      <x:c r="J6" s="9" t="str">
         <x:v>Trazabilidad ERP</x:v>
       </x:c>
     </x:row>
@@ -4079,16 +4341,20 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F7" s="3" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
-      </x:c>
-      <x:c r="G7" s="3" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="G7" s="10" t="str">
+        <x:v>XG-PRM-001 · Automatizado
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/promociones/XG-PRM-001.md</x:v>
+      </x:c>
+      <x:c r="H7" s="3" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H7" s="10" t="str">
+      <x:c r="I7" s="10" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I7" s="3" t="str">
+      <x:c r="J7" s="3" t="str">
         <x:v>test/ModuloFinanzas/Entidades/OfertaPorcentajeTest.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4110,16 +4376,20 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F8" s="7" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
-      </x:c>
-      <x:c r="G8" s="7" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="G8" s="11" t="str">
+        <x:v>XG-PRM-002 · Automatizado
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/promociones/XG-PRM-002.md</x:v>
+      </x:c>
+      <x:c r="H8" s="7" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H8" s="11" t="str">
+      <x:c r="I8" s="11" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I8" s="7" t="str">
+      <x:c r="J8" s="7" t="str">
         <x:v>test/ModuloFinanzas/Entidades/OfertaPrecioTest.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4141,16 +4411,20 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F9" s="3" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
-      </x:c>
-      <x:c r="G9" s="3" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="G9" s="10" t="str">
+        <x:v>XG-PRM-003 · Automatizado
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/promociones/XG-PRM-003.md</x:v>
+      </x:c>
+      <x:c r="H9" s="3" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H9" s="10" t="str">
+      <x:c r="I9" s="10" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I9" s="3" t="str">
+      <x:c r="J9" s="3" t="str">
         <x:v>test/ModuloFinanzas/Entidades/OfertaLlevaXPagaXTest.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4172,16 +4446,20 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F10" s="7" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
-      </x:c>
-      <x:c r="G10" s="7" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="G10" s="11" t="str">
+        <x:v>XG-PRM-004 · Automatizado
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/promociones/XG-PRM-004.md</x:v>
+      </x:c>
+      <x:c r="H10" s="7" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H10" s="11" t="str">
+      <x:c r="I10" s="11" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I10" s="7" t="str">
+      <x:c r="J10" s="7" t="str">
         <x:v>test/ModuloFinanzas/Entidades/OfertaCantidadPorcentajeTest.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4203,16 +4481,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F11" s="3" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G11" s="3" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H11" s="3" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H11" s="10" t="str">
+      <x:c r="I11" s="10" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I11" s="3" t="str">
+      <x:c r="J11" s="3" t="str">
         <x:v>test/ModuloFinanzas/Entidades/OfertaCantidadMayorPorcentajeTest.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4234,16 +4515,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F12" s="7" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G12" s="7" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H12" s="7" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H12" s="11" t="str">
+      <x:c r="I12" s="11" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I12" s="7" t="str">
+      <x:c r="J12" s="7" t="str">
         <x:v>test/ModuloFinanzas/Entidades/OfertaCantidadMayorImporteTest.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4265,16 +4549,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F13" s="3" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G13" s="3" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H13" s="3" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H13" s="10" t="str">
+      <x:c r="I13" s="10" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I13" s="3" t="str">
+      <x:c r="J13" s="3" t="str">
         <x:v>test/ModuloFinanzas/Entidades/OfertaCantidadMayorPrecioUnitarioTest.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4297,16 +4584,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F14" s="7" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G14" s="7" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H14" s="7" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H14" s="11" t="str">
+      <x:c r="I14" s="11" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I14" s="7" t="str">
+      <x:c r="J14" s="7" t="str">
         <x:v>test/ModuloFinanzas/Entidades/OfertaComboCalculadorTest.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4329,16 +4619,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F15" s="3" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G15" s="3" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H15" s="3" t="str">
         <x:v>Combo primero; 10% en A sobrante.</x:v>
       </x:c>
-      <x:c r="H15" s="10" t="str">
+      <x:c r="I15" s="10" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I15" s="3" t="str">
+      <x:c r="J15" s="3" t="str">
         <x:v>src/ModuloVentas/Servicios/OfertaComboService.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4360,16 +4653,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F16" s="7" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G16" s="7" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H16" s="7" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H16" s="11" t="str">
+      <x:c r="I16" s="11" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I16" s="7" t="str">
+      <x:c r="J16" s="7" t="str">
         <x:v>test/ModuloFinanzas/Entidades/OfertaPesableFraccionadoTest.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4391,16 +4687,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F17" s="3" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G17" s="3" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H17" s="3" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H17" s="10" t="str">
+      <x:c r="I17" s="10" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I17" s="3" t="str">
+      <x:c r="J17" s="3" t="str">
         <x:v>test/ModuloFinanzas/Entidades/OfertaPesableFraccionadoTest.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4422,16 +4721,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F18" s="7" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G18" s="7" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H18" s="7" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H18" s="11" t="str">
+      <x:c r="I18" s="11" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I18" s="7" t="str">
+      <x:c r="J18" s="7" t="str">
         <x:v>test/ModuloFinanzas/Entidades/OfertaPesableFraccionadoTest.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4455,16 +4757,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F19" s="3" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G19" s="3" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H19" s="3" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H19" s="10" t="str">
+      <x:c r="I19" s="10" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I19" s="3" t="str">
+      <x:c r="J19" s="3" t="str">
         <x:v>test/ModuloFinanzas/Entidades/OfertaAplicacionCalculadorAgrupacionTest.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4486,16 +4791,20 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F20" s="7" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
-      </x:c>
-      <x:c r="G20" s="7" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="G20" s="11" t="str">
+        <x:v>XG-PRM-005 · Automatizado
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/promociones/XG-PRM-005.md</x:v>
+      </x:c>
+      <x:c r="H20" s="7" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H20" s="11" t="str">
+      <x:c r="I20" s="11" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I20" s="7" t="str">
+      <x:c r="J20" s="7" t="str">
         <x:v>src/ModuloFinanzas/Entidades/OfertaLineaService.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4517,16 +4826,20 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F21" s="3" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
-      </x:c>
-      <x:c r="G21" s="3" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="G21" s="10" t="str">
+        <x:v>XG-PRM-006 · Automatizado
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/promociones/XG-PRM-006.md</x:v>
+      </x:c>
+      <x:c r="H21" s="3" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H21" s="10" t="str">
+      <x:c r="I21" s="10" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I21" s="3" t="str">
+      <x:c r="J21" s="3" t="str">
         <x:v>src/ModuloFinanzas/Entidades/OfertaLineaService.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4548,16 +4861,20 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F22" s="7" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
-      </x:c>
-      <x:c r="G22" s="7" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="G22" s="11" t="str">
+        <x:v>XG-PRM-007 · Automatizado
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/promociones/XG-PRM-007.md</x:v>
+      </x:c>
+      <x:c r="H22" s="7" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H22" s="11" t="str">
+      <x:c r="I22" s="11" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I22" s="7" t="str">
+      <x:c r="J22" s="7" t="str">
         <x:v>src/ModuloFinanzas/Entidades/OfertaLineaService.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4579,16 +4896,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F23" s="3" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G23" s="3" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H23" s="3" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H23" s="10" t="str">
+      <x:c r="I23" s="10" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I23" s="3" t="str">
+      <x:c r="J23" s="3" t="str">
         <x:v>src/ModuloFinanzas/Entidades/OfertaAplicacionCalculador.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4610,16 +4930,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F24" s="7" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G24" s="7" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H24" s="7" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H24" s="11" t="str">
+      <x:c r="I24" s="11" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I24" s="7" t="str">
+      <x:c r="J24" s="7" t="str">
         <x:v>src/ModuloFinanzas/Entidades/OfertaAplicacionCalculador.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4641,16 +4964,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F25" s="3" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G25" s="3" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H25" s="3" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H25" s="10" t="str">
+      <x:c r="I25" s="10" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I25" s="3" t="str">
+      <x:c r="J25" s="3" t="str">
         <x:v>src/ModuloFinanzas/Entidades/OfertaAplicacionCalculador.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4672,16 +4998,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F26" s="7" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G26" s="7" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H26" s="7" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H26" s="11" t="str">
+      <x:c r="I26" s="11" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I26" s="7" t="str">
+      <x:c r="J26" s="7" t="str">
         <x:v>src/ModuloFinanzas/Entidades/OfertaAplicacionCalculador.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4703,16 +5032,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F27" s="3" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G27" s="3" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H27" s="3" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H27" s="10" t="str">
+      <x:c r="I27" s="10" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I27" s="3" t="str">
+      <x:c r="J27" s="3" t="str">
         <x:v>src/ModuloProveedores/Entidades/ListaPrecioDetalle.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4734,16 +5066,19 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="F28" s="7" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G28" s="7" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H28" s="7" t="str">
         <x:v>Precio expresado en USD; conversión depende de la cotización del perfil.</x:v>
       </x:c>
-      <x:c r="H28" s="11" t="str">
+      <x:c r="I28" s="11" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I28" s="7" t="str">
+      <x:c r="J28" s="7" t="str">
         <x:v>src/ModuloProveedores/Entidades/ListaPrecioDetalle.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4765,16 +5100,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F29" s="3" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G29" s="3" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H29" s="3" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H29" s="10" t="str">
+      <x:c r="I29" s="10" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I29" s="3" t="str">
+      <x:c r="J29" s="3" t="str">
         <x:v>src/ModuloProveedores/Entidades/ListaPrecioDetalle.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4796,16 +5134,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F30" s="7" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G30" s="7" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H30" s="7" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H30" s="11" t="str">
+      <x:c r="I30" s="11" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I30" s="7" t="str">
+      <x:c r="J30" s="7" t="str">
         <x:v>src/ModuloProveedores/Entidades/ListaPrecioDetalle.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4827,16 +5168,19 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F31" s="3" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G31" s="3" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H31" s="3" t="str">
         <x:v>Ver condiciones del catálogo comercial.</x:v>
       </x:c>
-      <x:c r="H31" s="10" t="str">
+      <x:c r="I31" s="10" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I31" s="3" t="str">
+      <x:c r="J31" s="3" t="str">
         <x:v>src/ModuloProveedores/Entidades/ListaPrecioDetalle.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
@@ -4858,27 +5202,30 @@
         <x:v>ARS</x:v>
       </x:c>
       <x:c r="F32" s="7" t="str">
-        <x:v>Pendiente de ficha y automatización</x:v>
+        <x:v>Pendiente</x:v>
       </x:c>
       <x:c r="G32" s="7" t="str">
+        <x:v>Sin ficha</x:v>
+      </x:c>
+      <x:c r="H32" s="7" t="str">
         <x:v>La lista elegida contiene el producto y prevalece sobre el precio por cantidad.</x:v>
       </x:c>
-      <x:c r="H32" s="11" t="str">
+      <x:c r="I32" s="11" t="str">
         <x:v>Ver ejemplo
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/seeds/pricing.py</x:v>
       </x:c>
-      <x:c r="I32" s="7" t="str">
+      <x:c r="J32" s="7" t="str">
         <x:v>test/ModuloVentas/Vistas/FormVentaListaPrecioPrioridadPolicyTest.java
 Commit: f34238183d494259bed1279dd7d9aac0ce16a3ae</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A3:I4"/>
+    <x:mergeCell ref="A3:J4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2496d3a5835d47bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R052a0d1f048e4a45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
[feat] - Automatizar atajos de teclado en 13 listados
Agrega recorridos Robot y oráculos JAB para navegación, identidad, filtros y restricciones. Incorpora datos de ejemplo, pruebas sintéticas y actualiza el catálogo y el mapa de cobertura. La ejecución real del ERP sigue pendiente del paquete QA privado y la VM.
</commit_message>
<xml_diff>
--- a/docs/coverage/xgestion-cobertura.xlsx
+++ b/docs/coverage/xgestion-cobertura.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R6e624e07424446e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="2" r:id="Rf77db98947854cf7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenarios" sheetId="3" r:id="R49d39de9ccbe4bc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por detallar" sheetId="4" r:id="R597bfacc31344b4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplos seed" sheetId="5" r:id="Rcec29d9679904b46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R85ef3eb5bb894a4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="2" r:id="Rd506d7d597034665"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escenarios" sheetId="3" r:id="R6b9ee1f83dd64891"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por detallar" sheetId="4" r:id="Re2257c19a7b34e61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplos seed" sheetId="5" r:id="R4793f9cec9b743d6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -524,7 +524,7 @@
       </x:c>
       <x:c r="B8" s="21" t="n">
         <x:f>COUNTIF('Escenarios'!$C$7:$C$321,"Automatizado")</x:f>
-        <x:v>99</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C8" s="3" t="str">
         <x:v>Código de prueba disponible. Ejecución real pendiente.</x:v>
@@ -536,7 +536,7 @@
       </x:c>
       <x:c r="B9" s="22" t="n">
         <x:f>COUNTIF('Escenarios'!$C$7:$C$321,"Pendiente")</x:f>
-        <x:v>216</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
         <x:v>Criterios escritos; todavía sin prueba ejecutable.</x:v>
@@ -657,10 +657,10 @@
         <x:v>0. Preparación y ejecución comprensible</x:v>
       </x:c>
       <x:c r="B22" s="12" t="n">
-        <x:v>5</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C22" s="3" t="str">
-        <x:v>17 pendientes · 0 manuales</x:v>
+        <x:v>4 pendientes · 0 manuales</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
@@ -776,7 +776,7 @@
     </x:row>
     <x:row r="36" ht="28.5" customHeight="1">
       <x:c r="A36" s="7" t="str">
-        <x:v>Revisión de fuentes públicas: SHA256 182bd2ffb1ec0b45. Sin datos privados.</x:v>
+        <x:v>Revisión de fuentes públicas: SHA256 a6ce6d68a611f95b. Sin datos privados.</x:v>
       </x:c>
       <x:c r="B36" s="7"/>
       <x:c r="C36" s="7"/>
@@ -978,10 +978,10 @@
         <x:v>Reunir los escenarios implementados; no implica cubrir todo el ERP.</x:v>
       </x:c>
       <x:c r="E8" s="13" t="n">
-        <x:v>99</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="F8" s="13" t="n">
-        <x:v>216</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="G8" s="13" t="n">
         <x:v>0</x:v>
@@ -3189,7 +3189,7 @@
         <x:v>XG-FIN-011..014</x:v>
       </x:c>
     </x:row>
-    <x:row r="82" ht="40.5" customHeight="1">
+    <x:row r="82" ht="54" customHeight="1">
       <x:c r="A82" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -3200,19 +3200,19 @@
         <x:v>atajos-listados</x:v>
       </x:c>
       <x:c r="D82" s="7" t="str">
-        <x:v>13 recorridos pendientes de teclado, identidad, búsqueda, orden y restricciones.</x:v>
+        <x:v>13 recorridos automatizados de teclado, identidad, búsqueda, orden y restricciones; validación JAB pendiente.</x:v>
       </x:c>
       <x:c r="E82" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F82" s="13" t="n">
-        <x:v>13</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G82" s="13" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H82" s="7" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Parcial: ejecutable</x:v>
       </x:c>
       <x:c r="I82" s="7" t="str">
         <x:v>XG-KEY-001..013</x:v>
@@ -3229,19 +3229,19 @@
         <x:v>filtros-listados</x:v>
       </x:c>
       <x:c r="D83" s="3" t="str">
-        <x:v>Ocho modales pendientes: foco, borrador, aplicar una vez y cancelar por cada salida.</x:v>
+        <x:v>Ocho recorridos automatizados de filtros; validación JAB pendiente.</x:v>
       </x:c>
       <x:c r="E83" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F83" s="12" t="n">
-        <x:v>8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G83" s="12" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H83" s="3" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Parcial: ejecutable</x:v>
       </x:c>
       <x:c r="I83" s="3" t="str">
         <x:v>XG-KEY-001..004, XG-KEY-006..007, XG-KEY-010
@@ -3254,7 +3254,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c42cef8243b42b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R588f4ba088eb4b93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6740,7 +6740,7 @@
         <x:v>Atajos en cuentas corrientes de clientes</x:v>
       </x:c>
       <x:c r="C98" s="7" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D98" s="7" t="str">
         <x:v>Pendiente</x:v>
@@ -6760,11 +6760,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/atajos-listados/XG-KEY-001.md</x:v>
       </x:c>
-      <x:c r="I98" s="7" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I98" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/atajos_listados.robot</x:v>
       </x:c>
       <x:c r="J98" s="7" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="67.5" customHeight="1">
@@ -6775,7 +6776,7 @@
         <x:v>Atajos en cuenta corriente de cliente</x:v>
       </x:c>
       <x:c r="C99" s="3" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D99" s="3" t="str">
         <x:v>Pendiente</x:v>
@@ -6795,11 +6796,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/atajos-listados/XG-KEY-002.md</x:v>
       </x:c>
-      <x:c r="I99" s="3" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I99" s="10" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/atajos_listados.robot</x:v>
       </x:c>
       <x:c r="J99" s="3" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="67.5" customHeight="1">
@@ -6810,7 +6812,7 @@
         <x:v>Atajos en cuentas corrientes de proveedores</x:v>
       </x:c>
       <x:c r="C100" s="7" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D100" s="7" t="str">
         <x:v>Pendiente</x:v>
@@ -6830,11 +6832,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/atajos-listados/XG-KEY-003.md</x:v>
       </x:c>
-      <x:c r="I100" s="7" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I100" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/atajos_listados.robot</x:v>
       </x:c>
       <x:c r="J100" s="7" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="67.5" customHeight="1">
@@ -6845,7 +6848,7 @@
         <x:v>Atajos en cuenta corriente de proveedor</x:v>
       </x:c>
       <x:c r="C101" s="3" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D101" s="3" t="str">
         <x:v>Pendiente</x:v>
@@ -6865,11 +6868,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/atajos-listados/XG-KEY-004.md</x:v>
       </x:c>
-      <x:c r="I101" s="3" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I101" s="10" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/atajos_listados.robot</x:v>
       </x:c>
       <x:c r="J101" s="3" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="67.5" customHeight="1">
@@ -6880,7 +6884,7 @@
         <x:v>Atajos en clientes</x:v>
       </x:c>
       <x:c r="C102" s="7" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D102" s="7" t="str">
         <x:v>Pendiente</x:v>
@@ -6899,11 +6903,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/atajos-listados/XG-KEY-005.md</x:v>
       </x:c>
-      <x:c r="I102" s="7" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I102" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/atajos_listados.robot</x:v>
       </x:c>
       <x:c r="J102" s="7" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="67.5" customHeight="1">
@@ -6914,7 +6919,7 @@
         <x:v>Atajos en productos</x:v>
       </x:c>
       <x:c r="C103" s="3" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D103" s="3" t="str">
         <x:v>Pendiente</x:v>
@@ -6934,11 +6939,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/atajos-listados/XG-KEY-006.md</x:v>
       </x:c>
-      <x:c r="I103" s="3" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I103" s="10" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/atajos_listados.robot</x:v>
       </x:c>
       <x:c r="J103" s="3" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="67.5" customHeight="1">
@@ -6949,7 +6955,7 @@
         <x:v>Atajos en mesas</x:v>
       </x:c>
       <x:c r="C104" s="7" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D104" s="7" t="str">
         <x:v>Pendiente</x:v>
@@ -6969,11 +6975,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/atajos-listados/XG-KEY-007.md</x:v>
       </x:c>
-      <x:c r="I104" s="7" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I104" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/atajos_listados.robot</x:v>
       </x:c>
       <x:c r="J104" s="7" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="67.5" customHeight="1">
@@ -6984,7 +6991,7 @@
         <x:v>Atajos en usuarios</x:v>
       </x:c>
       <x:c r="C105" s="3" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D105" s="3" t="str">
         <x:v>Pendiente</x:v>
@@ -7003,11 +7010,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/atajos-listados/XG-KEY-008.md</x:v>
       </x:c>
-      <x:c r="I105" s="3" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I105" s="10" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/atajos_listados.robot</x:v>
       </x:c>
       <x:c r="J105" s="3" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="67.5" customHeight="1">
@@ -7018,7 +7026,7 @@
         <x:v>Atajos en turnos</x:v>
       </x:c>
       <x:c r="C106" s="7" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D106" s="7" t="str">
         <x:v>Pendiente</x:v>
@@ -7037,11 +7045,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/atajos-listados/XG-KEY-009.md</x:v>
       </x:c>
-      <x:c r="I106" s="7" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I106" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/atajos_listados.robot</x:v>
       </x:c>
       <x:c r="J106" s="7" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="67.5" customHeight="1">
@@ -7052,7 +7061,7 @@
         <x:v>Atajos en compras</x:v>
       </x:c>
       <x:c r="C107" s="3" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D107" s="3" t="str">
         <x:v>Pendiente</x:v>
@@ -7072,11 +7081,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/atajos-listados/XG-KEY-010.md</x:v>
       </x:c>
-      <x:c r="I107" s="3" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I107" s="10" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/atajos_listados.robot</x:v>
       </x:c>
       <x:c r="J107" s="3" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="67.5" customHeight="1">
@@ -7087,7 +7097,7 @@
         <x:v>Atajos en proveedores</x:v>
       </x:c>
       <x:c r="C108" s="7" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D108" s="7" t="str">
         <x:v>Pendiente</x:v>
@@ -7106,11 +7116,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/atajos-listados/XG-KEY-011.md</x:v>
       </x:c>
-      <x:c r="I108" s="7" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I108" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/atajos_listados.robot</x:v>
       </x:c>
       <x:c r="J108" s="7" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="67.5" customHeight="1">
@@ -7121,7 +7132,7 @@
         <x:v>Atajos en categorías</x:v>
       </x:c>
       <x:c r="C109" s="3" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D109" s="3" t="str">
         <x:v>Pendiente</x:v>
@@ -7140,11 +7151,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/atajos-listados/XG-KEY-012.md</x:v>
       </x:c>
-      <x:c r="I109" s="3" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I109" s="10" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/atajos_listados.robot</x:v>
       </x:c>
       <x:c r="J109" s="3" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="67.5" customHeight="1">
@@ -7155,7 +7167,7 @@
         <x:v>Atajos en subcategorías</x:v>
       </x:c>
       <x:c r="C110" s="7" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Automatizado</x:v>
       </x:c>
       <x:c r="D110" s="7" t="str">
         <x:v>Pendiente</x:v>
@@ -7175,11 +7187,12 @@
         <x:v>Ver ficha
 https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/scenarios/atajos-listados/XG-KEY-013.md</x:v>
       </x:c>
-      <x:c r="I110" s="7" t="str">
-        <x:v>Sin automatizar</x:v>
+      <x:c r="I110" s="11" t="str">
+        <x:v>Ver prueba
+https://github.com/darioravello89/xsoft-qa-e2e/blob/main/products/xgestion/suites/atajos_listados.robot</x:v>
       </x:c>
       <x:c r="J110" s="7" t="str">
-        <x:v>Implementar la ficha y luego validar sobre el JAR QA.</x:v>
+        <x:v>Calibrar y ejecutar sobre el JAR QA; registrar evidencia.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="67.5" customHeight="1">
@@ -14954,7 +14967,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39be5d36afd343c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ab24b2452d9487b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16301,7 +16314,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd1fbb69fdea4d16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d3c0c971a424470"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17341,7 +17354,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d039d305efb4478"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb72b5bdb4c7c4a42"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>